<commit_message>
Add updated Bloom verbs lexicon and fix various files
- Updated the "Stavfel och språkbruk.md" file to reflect the correct number of findings and adjusted the download link for the Excel file.
- Added new Python script "bloom_verbs.py" containing a comprehensive lexicon of Bloom's taxonomy verbs in Swedish, categorized by cognitive levels.
- Updated several Excel files in the analysis directory, indicating differences in their binary content.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Bloom-taxonomi.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Bloom-taxonomi.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Bloom-taxonomi" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bloom-taxonomi'!$A$1:$E$24</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -462,7 +469,677 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ABY22W</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BYA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [2,1,2,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY22W</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>BFY226</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FYA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Okänt ledande verb</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3 av 12 bullets har okänt ledande verb</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY226</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>GIK299</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Okänt ledande verb</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>4 av 11 bullets har okänt ledande verb</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK299</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GIK2PG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,0,2,1]</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>GIK38J</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [0,1,0,0,1,1]</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38J</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>GMD2PA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MDI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Okänt ledande verb</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3 av 6 bullets har okänt ledande verb</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,0,1,1]</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>AEG225</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,0,1,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>AEG2AK</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,2,2,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AEG2AP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [2,1,1,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AEG2AQ</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,3,0,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>AEG2B6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [2,1,2,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>EG3015</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [2,2,1,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EG3019</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [1,2,2,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3019</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>EG3020</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [6,0,0,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>EG3022</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [8,0,0,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>GEG26J</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [0,0,0,1,0,2]</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>GEG3DV</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [1,0,0,1,2,1]</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3DV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>GSQ25F</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [0,0,0,1,0,2]</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2VY</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [2,0,0,0,1,2]</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>AMI22Z</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [2,0,3,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>AMI23A</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Låg verbnivå för avancerad kurs</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Avancerad kurs utan analysera/värdera/skapa-verb; fördelning [2,1,1,0,0,0]</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>GMI24H</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Hög verbnivå för grundkurs</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Grundkurs domineras av värdera/skapa; fördelning [0,0,1,0,1,1]</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:E24"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>